<commit_message>
Erweitere den Beförderungsrechner auf mehrere Ämter und die Auswahl vom November 2026.
Die Wartezeiten der zweiten und dritten Qualifikationsebene folgen der BefRPolVS; A 9 mit Amtszulage behält die Beförderungsauswahl. Das Personalrat-Signet ersetzt den Polizeistern.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Beförderungswahl zum A9Z.xlsx
+++ b/Beförderungswahl zum A9Z.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Antigravity\Tool zum Berechnen zum A9Z\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D9A2641-4C13-4713-B751-8CE0C237251D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC1623DD-CD0C-4F56-ADF5-55DCD98A16B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19118" yWindow="0" windowWidth="19365" windowHeight="20963" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Beförderungsauswahl" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="75">
   <si>
     <t>Stichtag</t>
   </si>
@@ -242,13 +242,16 @@
   </si>
   <si>
     <t>DZ in A 9 mind. 104 Mon. ODER allg. DZ mind. 188 Mon.</t>
+  </si>
+  <si>
+    <t>DZ in A 9 mind. 87 Monate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -277,6 +280,11 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -548,16 +556,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="9.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" customWidth="1"/>
-    <col min="5" max="5" width="39.140625" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" customWidth="1"/>
-    <col min="7" max="7" width="8.28515625" customWidth="1"/>
+    <col min="1" max="1" width="14.73046875" customWidth="1"/>
+    <col min="2" max="2" width="11.3984375" customWidth="1"/>
+    <col min="3" max="3" width="9.3984375" customWidth="1"/>
+    <col min="4" max="4" width="14.3984375" customWidth="1"/>
+    <col min="5" max="5" width="39.1328125" customWidth="1"/>
+    <col min="6" max="6" width="9.3984375" customWidth="1"/>
+    <col min="7" max="7" width="8.265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="38.25" customHeight="1" thickBot="1">
@@ -583,7 +591,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="13.5" thickBot="1">
+    <row r="2" spans="1:7" ht="13.15" thickBot="1">
       <c r="A2" s="7">
         <v>45170</v>
       </c>
@@ -606,7 +614,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="13.5" thickBot="1">
+    <row r="3" spans="1:7" ht="13.15" thickBot="1">
       <c r="A3" s="7">
         <v>45200</v>
       </c>
@@ -629,7 +637,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="13.5" thickBot="1">
+    <row r="4" spans="1:7" ht="13.15" thickBot="1">
       <c r="A4" s="7">
         <v>45231</v>
       </c>
@@ -652,7 +660,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="13.5" thickBot="1">
+    <row r="5" spans="1:7" ht="13.15" thickBot="1">
       <c r="A5" s="7">
         <v>45261</v>
       </c>
@@ -675,7 +683,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="13.5" thickBot="1">
+    <row r="6" spans="1:7" ht="13.15" thickBot="1">
       <c r="A6" s="7">
         <v>45292</v>
       </c>
@@ -698,7 +706,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="13.5" thickBot="1">
+    <row r="7" spans="1:7" ht="13.15" thickBot="1">
       <c r="A7" s="7">
         <v>45323</v>
       </c>
@@ -721,7 +729,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="13.5" thickBot="1">
+    <row r="8" spans="1:7" ht="13.15" thickBot="1">
       <c r="A8" s="7">
         <v>45352</v>
       </c>
@@ -744,7 +752,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="13.5" thickBot="1">
+    <row r="9" spans="1:7" ht="13.15" thickBot="1">
       <c r="A9" s="7">
         <v>45383</v>
       </c>
@@ -767,7 +775,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="13.5" thickBot="1">
+    <row r="10" spans="1:7" ht="13.15" thickBot="1">
       <c r="A10" s="7">
         <v>45413</v>
       </c>
@@ -790,7 +798,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="13.5" thickBot="1">
+    <row r="11" spans="1:7" ht="13.15" thickBot="1">
       <c r="A11" s="7">
         <v>45444</v>
       </c>
@@ -813,7 +821,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="13.5" thickBot="1">
+    <row r="12" spans="1:7" ht="13.15" thickBot="1">
       <c r="A12" s="7">
         <v>45474</v>
       </c>
@@ -836,7 +844,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="13.5" thickBot="1">
+    <row r="13" spans="1:7" ht="13.15" thickBot="1">
       <c r="A13" s="7">
         <v>45505</v>
       </c>
@@ -859,7 +867,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="13.5" thickBot="1">
+    <row r="14" spans="1:7" ht="13.15" thickBot="1">
       <c r="A14" s="7">
         <v>45536</v>
       </c>
@@ -882,7 +890,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="13.5" thickBot="1">
+    <row r="15" spans="1:7" ht="13.15" thickBot="1">
       <c r="A15" s="7">
         <v>45566</v>
       </c>
@@ -905,7 +913,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="13.5" thickBot="1">
+    <row r="16" spans="1:7" ht="13.15" thickBot="1">
       <c r="A16" s="7">
         <v>45597</v>
       </c>
@@ -928,7 +936,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="13.5" thickBot="1">
+    <row r="17" spans="1:7" ht="13.15" thickBot="1">
       <c r="A17" s="7">
         <v>45627</v>
       </c>
@@ -951,7 +959,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="13.5" thickBot="1">
+    <row r="18" spans="1:7" ht="13.15" thickBot="1">
       <c r="A18" s="7">
         <v>45658</v>
       </c>
@@ -974,7 +982,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="13.5" thickBot="1">
+    <row r="19" spans="1:7" ht="13.15" thickBot="1">
       <c r="A19" s="7">
         <v>45689</v>
       </c>
@@ -997,7 +1005,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="13.5" thickBot="1">
+    <row r="20" spans="1:7" ht="13.15" thickBot="1">
       <c r="A20" s="7">
         <v>45717</v>
       </c>
@@ -1020,7 +1028,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="13.5" thickBot="1">
+    <row r="21" spans="1:7" ht="13.15" thickBot="1">
       <c r="A21" s="7">
         <v>45748</v>
       </c>
@@ -1043,7 +1051,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="13.5" thickBot="1">
+    <row r="22" spans="1:7" ht="13.15" thickBot="1">
       <c r="A22" s="7">
         <v>45778</v>
       </c>
@@ -1066,7 +1074,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="13.5" thickBot="1">
+    <row r="23" spans="1:7" ht="13.15" thickBot="1">
       <c r="A23" s="7">
         <v>45809</v>
       </c>
@@ -1089,7 +1097,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="13.5" thickBot="1">
+    <row r="24" spans="1:7" ht="13.15" thickBot="1">
       <c r="A24" s="7">
         <v>45839</v>
       </c>
@@ -1112,7 +1120,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="13.5" thickBot="1">
+    <row r="25" spans="1:7" ht="13.15" thickBot="1">
       <c r="A25" s="7">
         <v>45870</v>
       </c>
@@ -1135,7 +1143,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="13.5" thickBot="1">
+    <row r="26" spans="1:7" ht="13.15" thickBot="1">
       <c r="A26" s="7">
         <v>45901</v>
       </c>
@@ -1158,7 +1166,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="13.5" thickBot="1">
+    <row r="27" spans="1:7" ht="13.15" thickBot="1">
       <c r="A27" s="7">
         <v>45931</v>
       </c>
@@ -1181,7 +1189,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="13.5" thickBot="1">
+    <row r="28" spans="1:7" ht="13.15" thickBot="1">
       <c r="A28" s="7">
         <v>45962</v>
       </c>
@@ -1204,7 +1212,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="13.5" thickBot="1">
+    <row r="29" spans="1:7" ht="13.15" thickBot="1">
       <c r="A29" s="7">
         <v>45992</v>
       </c>
@@ -1227,7 +1235,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="13.5" thickBot="1">
+    <row r="30" spans="1:7" ht="13.15" thickBot="1">
       <c r="A30" s="7">
         <v>46023</v>
       </c>
@@ -1250,7 +1258,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="13.5" thickBot="1">
+    <row r="31" spans="1:7" ht="13.15" thickBot="1">
       <c r="A31" s="7">
         <v>46054</v>
       </c>
@@ -1273,7 +1281,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="13.5" thickBot="1">
+    <row r="32" spans="1:7" ht="13.15" thickBot="1">
       <c r="A32" s="7">
         <v>46082</v>
       </c>
@@ -1296,7 +1304,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="13.5" thickBot="1">
+    <row r="33" spans="1:7" ht="13.15" thickBot="1">
       <c r="A33" s="7">
         <v>46113</v>
       </c>
@@ -1319,7 +1327,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="13.5" thickBot="1">
+    <row r="34" spans="1:7" ht="13.15" thickBot="1">
       <c r="A34" s="7">
         <v>46143</v>
       </c>
@@ -1342,7 +1350,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="13.5" thickBot="1">
+    <row r="35" spans="1:7" ht="13.15" thickBot="1">
       <c r="A35" s="7">
         <v>46174</v>
       </c>
@@ -1365,7 +1373,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="13.5" thickBot="1">
+    <row r="36" spans="1:7" ht="13.15" thickBot="1">
       <c r="A36" s="7">
         <v>46204</v>
       </c>
@@ -1388,7 +1396,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="13.5" thickBot="1">
+    <row r="37" spans="1:7" ht="13.15" thickBot="1">
       <c r="A37" s="7">
         <v>46235</v>
       </c>
@@ -1411,7 +1419,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="13.5" thickBot="1">
+    <row r="38" spans="1:7" ht="13.15" thickBot="1">
       <c r="A38" s="7">
         <v>46266</v>
       </c>
@@ -1434,7 +1442,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="13.5" thickBot="1">
+    <row r="39" spans="1:7" ht="13.15" thickBot="1">
       <c r="A39" s="7">
         <v>46296</v>
       </c>
@@ -1457,7 +1465,58 @@
         <v>35</v>
       </c>
     </row>
+    <row r="40" spans="1:7" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A40" s="7">
+        <v>46327</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F40" s="4">
+        <v>1966</v>
+      </c>
+      <c r="G40" s="5">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A41" s="7"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="5"/>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A42" s="7"/>
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="5"/>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A43" s="7"/>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="5"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>